<commit_message>
commit - 11 (Test Run)
</commit_message>
<xml_diff>
--- a/qa-artifacts/FoodHub-AI-Test-Analysis.xlsx
+++ b/qa-artifacts/FoodHub-AI-Test-Analysis.xlsx
@@ -400,19 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J4"/>
-  <cols>
-    <col min="1" max="1" width="13.83203125" customWidth="1"/>
-    <col min="2" max="2" width="27.83203125" customWidth="1"/>
-    <col min="3" max="3" width="64.83203125" customWidth="1"/>
-    <col min="4" max="4" width="49.83203125" customWidth="1"/>
-    <col min="5" max="5" width="53.83203125" customWidth="1"/>
-    <col min="6" max="6" width="31.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="58.83203125" customWidth="1"/>
-    <col min="9" max="9" width="43.83203125" customWidth="1"/>
-    <col min="10" max="10" width="48.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:J6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -448,125 +436,174 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>AI-FAIL-001</v>
+        <v>FOL-001</v>
       </c>
       <c r="B2" t="str">
-        <v>Log capture</v>
+        <v>E2E Tests (Playwright)</v>
       </c>
       <c r="C2" t="str">
-        <v>Vitest, Pact, Playwright, Testcontainers, k6, and viewer logs retained</v>
+        <v>Timeout</v>
       </c>
       <c r="D2" t="str">
-        <v>Test logs and generated reports</v>
+        <v>2 occurrences: 'expect(locator).toHaveText: Timeout 5000ms exceeded' on #gateway-message; expected 'Payment declined for xxxx-xxxx-xxxx-8911.' but received 'Processing through FoodHub Payment Gateway...'</v>
       </c>
       <c r="E2" t="str">
-        <v>Unknown until logs are analyzed</v>
+        <v>Gateway UI update delayed; test assertion runs before the final 'declined' message replaces the processing state</v>
       </c>
       <c r="F2" t="str">
-        <v>Unknown</v>
+        <v>test</v>
       </c>
       <c r="G2" t="str">
-        <v>Medium</v>
+        <v>medium</v>
       </c>
       <c r="H2" t="str">
-        <v>Run analyzer and compare against observability artifacts</v>
+        <v>Replace immediate toHaveText with web-first assertions (waitForSelector with state 'attached' or 'visible') or poll for the expected final text with a generous timeout</v>
       </c>
       <c r="I2" t="str">
-        <v>Local fallback</v>
+        <v>sample-flaky-log.txt</v>
       </c>
       <c r="J2" t="str">
-        <v>deepseek-v4-pro high when FOODHUB_AI_LIVE=true</v>
+        <v>DeepSeek</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>AI-FAIL-002</v>
+        <v>FOL-002</v>
       </c>
       <c r="B3" t="str">
-        <v>Pattern analysis</v>
+        <v>E2E Tests (Playwright)</v>
       </c>
       <c r="C3" t="str">
-        <v>Timeout, selector, startup, Pact, DB, and k6 signals scanned</v>
+        <v>Selector / UI locator</v>
       </c>
       <c r="D3" t="str">
-        <v>tests/fixtures/failureLogs/sample-flaky-log.txt</v>
+        <v>3 occurrences: locator '#gateway-message' text mismatch; received 'Processing through FoodHub Payment Gateway...' instead of expected declined message</v>
       </c>
       <c r="E3" t="str">
-        <v>Potential flaky test or environment issue</v>
+        <v>Locator is too generic; same element updates asynchronously during payment flow, causing assertion on intermediate state</v>
       </c>
       <c r="F3" t="str">
-        <v>Test or Environment</v>
+        <v>test</v>
       </c>
       <c r="G3" t="str">
-        <v>Medium</v>
+        <v>medium</v>
       </c>
       <c r="H3" t="str">
-        <v>Classify each hit and attach next diagnostic command</v>
+        <v>Use a more specific locator for the final declined message (e.g., text='Payment declined') or wait until the element contains the exact string before asserting</v>
       </c>
       <c r="I3" t="str">
-        <v>Local fallback</v>
+        <v>sample-flaky-log.txt</v>
       </c>
       <c r="J3" t="str">
-        <v>deepseek-v4-pro high when FOODHUB_AI_LIVE=true</v>
+        <v>DeepSeek</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>AI-FAIL-003</v>
+        <v>FOL-003</v>
       </c>
       <c r="B4" t="str">
-        <v>Observability correlation</v>
+        <v>E2E Tests (Playwright)</v>
       </c>
       <c r="C4" t="str">
-        <v>Failure details compared with Firebase run history and request logs</v>
+        <v>Network / service startup</v>
       </c>
       <c r="D4" t="str">
-        <v>FoodHub-Observability-Dashboard.xlsx</v>
+        <v>1 occurrence: 'page.goto: net::ERR_CONNECTION_REFUSED at http://127.0.0.1:4173/'</v>
       </c>
       <c r="E4" t="str">
-        <v>Request-level regression or missing metric evidence</v>
+        <v>FoodHub app (port 4173) not listening when Playwright test starts; no startup health check performed</v>
       </c>
       <c r="F4" t="str">
-        <v>Product, Test, or Environment</v>
+        <v>environment</v>
       </c>
       <c r="G4" t="str">
-        <v>Medium</v>
+        <v>high</v>
       </c>
       <c r="H4" t="str">
-        <v>Correlate failed test timestamp with request logs</v>
+        <v>Add a pre-test step (e.g., wait-on http://127.0.0.1:4173/health or Playwright's webServer config with reuseExistingServer) to guarantee the app is ready before each e2e run</v>
       </c>
       <c r="I4" t="str">
-        <v>deepseek-v4-pro when live mode is enabled</v>
+        <v>sample-flaky-log.txt</v>
       </c>
       <c r="J4" t="str">
-        <v>deepseek-v4-pro high when FOODHUB_AI_LIVE=true</v>
+        <v>DeepSeek</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>FOL-004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>E2E Tests (Playwright)</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Payment gateway flow</v>
+      </c>
+      <c r="D5" t="str">
+        <v>10 occurrences across logged tests: redirect to gateway, payment processing, and message updates are brittle; one case timed out waiting for 'declined' message</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Synchronization issues between FoodHub and Payment Gateway; gateway callback or UI update may be slow, causing tests to observe intermediate processing states</v>
+      </c>
+      <c r="F5" t="str">
+        <v>environment</v>
+      </c>
+      <c r="G5" t="str">
+        <v>medium</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Wait for the gateway's final processing before asserting (e.g., waitForURL that returns to FoodHub, or waitForResponse on the order API before checking UI); verify gateway health as part of setup</v>
+      </c>
+      <c r="I5" t="str">
+        <v>sample-flaky-log.txt</v>
+      </c>
+      <c r="J5" t="str">
+        <v>DeepSeek</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>FOL-005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>E2E Tests (Playwright)</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Retry signal</v>
+      </c>
+      <c r="D6" t="str">
+        <v>1 occurrence: test 'customer can view menu, pay through the gateway, and receive an AI suggestion' failed with ERR_CONNECTION_REFUSED, then passed on Retry #1</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Environment not ready for initial attempt; retry succeeds only after the app fully starts</v>
+      </c>
+      <c r="F6" t="str">
+        <v>environment</v>
+      </c>
+      <c r="G6" t="str">
+        <v>high</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Remove dependency on retries by ensuring pre-test health checks; if retries are kept, investigate the exact readiness gap and add an explicit wait before the first navigation</v>
+      </c>
+      <c r="I6" t="str">
+        <v>sample-flaky-log.txt</v>
+      </c>
+      <c r="J6" t="str">
+        <v>DeepSeek</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M12"/>
-  <cols>
-    <col min="1" max="1" width="13.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="64.83203125" customWidth="1"/>
-    <col min="5" max="5" width="55.83203125" customWidth="1"/>
-    <col min="6" max="6" width="13.83203125" customWidth="1"/>
-    <col min="7" max="7" width="64.83203125" customWidth="1"/>
-    <col min="8" max="8" width="33.83203125" customWidth="1"/>
-    <col min="9" max="9" width="13.83203125" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="7.83203125" customWidth="1"/>
-    <col min="12" max="12" width="15.83203125" customWidth="1"/>
-    <col min="13" max="13" width="38.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:M16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -611,31 +648,31 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>AI-EDGE-001</v>
+        <v>FH-EDGE-001</v>
       </c>
       <c r="B2" t="str">
         <v>Edge Case</v>
       </c>
       <c r="C2" t="str">
-        <v>Menu</v>
+        <v>API</v>
       </c>
       <c r="D2" t="str">
-        <v>Menu API returns stable item contract</v>
+        <v>POST /order with negative quantity for a menu item</v>
       </c>
       <c r="E2" t="str">
-        <v>API contract breaking</v>
+        <v>Validation might not reject negative integer quantity, leading to incorrect pricing or downstream errors</v>
       </c>
       <c r="F2" t="str">
         <v>Integration</v>
       </c>
       <c r="G2" t="str">
-        <v>GET /menu returns items with id, name, price, and category</v>
+        <v>Response status 400 with error 'Invalid order'</v>
       </c>
       <c r="H2" t="str">
-        <v>Menu response fixture</v>
+        <v>Payload with items: [{ menuItemId: 'burger-classic', quantity: -1 }], valid paymentToken and customerName</v>
       </c>
       <c r="I2" t="str">
-        <v>Implemented</v>
+        <v>To Do</v>
       </c>
       <c r="J2" t="str">
         <v/>
@@ -644,39 +681,39 @@
         <v/>
       </c>
       <c r="L2" t="str">
-        <v/>
+        <v>AI-generated</v>
       </c>
       <c r="M2" t="str">
-        <v>Fallback unless FOODHUB_AI_LIVE=true</v>
+        <v>DeepSeek</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>AI-EDGE-002</v>
+        <v>FH-EDGE-002</v>
       </c>
       <c r="B3" t="str">
         <v>Edge Case</v>
       </c>
       <c r="C3" t="str">
-        <v>Order</v>
+        <v>API</v>
       </c>
       <c r="D3" t="str">
-        <v>Order contains an unknown menu item</v>
+        <v>POST /order with zero quantity for a menu item</v>
       </c>
       <c r="E3" t="str">
-        <v>Invalid menu items</v>
+        <v>Zero quantity should be rejected per business logic but may pass validation</v>
       </c>
       <c r="F3" t="str">
         <v>Integration</v>
       </c>
       <c r="G3" t="str">
-        <v>POST /order returns 400 Invalid order</v>
+        <v>Response status 400 with error 'Invalid order'</v>
       </c>
       <c r="H3" t="str">
-        <v>Unknown item id payload</v>
+        <v>Payload with items: [{ menuItemId: 'burger-classic', quantity: 0 }], valid paymentToken and customerName</v>
       </c>
       <c r="I3" t="str">
-        <v>Implemented</v>
+        <v>To Do</v>
       </c>
       <c r="J3" t="str">
         <v/>
@@ -685,39 +722,39 @@
         <v/>
       </c>
       <c r="L3" t="str">
-        <v/>
+        <v>AI-generated</v>
       </c>
       <c r="M3" t="str">
-        <v>Fallback unless FOODHUB_AI_LIVE=true</v>
+        <v>DeepSeek</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>AI-EDGE-003</v>
+        <v>FH-EDGE-003</v>
       </c>
       <c r="B4" t="str">
         <v>Edge Case</v>
       </c>
       <c r="C4" t="str">
-        <v>Order</v>
+        <v>API</v>
       </c>
       <c r="D4" t="str">
-        <v>Order contains no items</v>
+        <v>POST /order with non-integer quantity (e.g., 1.5)</v>
       </c>
       <c r="E4" t="str">
-        <v>Invalid empty orders</v>
+        <v>Zod schema int validation might accept if coerced? Should reject.</v>
       </c>
       <c r="F4" t="str">
         <v>Integration</v>
       </c>
       <c r="G4" t="str">
-        <v>POST /order returns 400 with empty-order detail</v>
+        <v>Response status 400 with error 'Invalid order'</v>
       </c>
       <c r="H4" t="str">
-        <v>Empty items payload</v>
+        <v>Payload with items: [{ menuItemId: 'burger-classic', quantity: 1.5 }], valid paymentToken and customerName</v>
       </c>
       <c r="I4" t="str">
-        <v>Implemented</v>
+        <v>To Do</v>
       </c>
       <c r="J4" t="str">
         <v/>
@@ -726,39 +763,39 @@
         <v/>
       </c>
       <c r="L4" t="str">
-        <v/>
+        <v>AI-generated</v>
       </c>
       <c r="M4" t="str">
-        <v>Fallback unless FOODHUB_AI_LIVE=true</v>
+        <v>DeepSeek</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>AI-EDGE-004</v>
+        <v>FH-EDGE-004</v>
       </c>
       <c r="B5" t="str">
         <v>Edge Case</v>
       </c>
       <c r="C5" t="str">
-        <v>Totals</v>
+        <v>API</v>
       </c>
       <c r="D5" t="str">
-        <v>Order has mixed item quantities and decimal prices</v>
+        <v>POST /order with quantity exceeding upper boundary (21)</v>
       </c>
       <c r="E5" t="str">
-        <v>Incorrect totals</v>
+        <v>Boundary check at 20 may be missed, leading to order creation with excessive quantity</v>
       </c>
       <c r="F5" t="str">
-        <v>Unit</v>
+        <v>Integration</v>
       </c>
       <c r="G5" t="str">
-        <v>Total is rounded to two decimals and payment is charged once</v>
+        <v>Response status 400 with error 'Invalid order'</v>
       </c>
       <c r="H5" t="str">
-        <v>Mixed quantity order builder</v>
+        <v>Payload with items: [{ menuItemId: 'burger-classic', quantity: 21 }], valid paymentToken and customerName</v>
       </c>
       <c r="I5" t="str">
-        <v>Implemented</v>
+        <v>To Do</v>
       </c>
       <c r="J5" t="str">
         <v/>
@@ -767,261 +804,261 @@
         <v/>
       </c>
       <c r="L5" t="str">
-        <v/>
+        <v>AI-generated</v>
       </c>
       <c r="M5" t="str">
-        <v>Fallback unless FOODHUB_AI_LIVE=true</v>
+        <v>DeepSeek</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>AI-EDGE-005</v>
+        <v>FH-MISS-001</v>
       </c>
       <c r="B6" t="str">
-        <v>Edge Case</v>
+        <v>Missing Scenario</v>
       </c>
       <c r="C6" t="str">
-        <v>Invoice</v>
+        <v>UI</v>
       </c>
       <c r="D6" t="str">
-        <v>Paid order invoice link shows transaction, order, card last 4, paid-via, and customer name</v>
+        <v>Customer sees error message when payment gateway is unreachable</v>
       </c>
       <c r="E6" t="str">
-        <v>Receipt/invoice evidence missing</v>
+        <v>User receives no feedback or a generic error when gateway is down, causing confusion</v>
       </c>
       <c r="F6" t="str">
         <v>E2E</v>
       </c>
       <c r="G6" t="str">
-        <v>Invoice panel opens from last transaction link and matches payment gateway data</v>
+        <v>Appropriate error message displayed (e.g., 'FoodHub Payment Gateway unavailable'), user can retry</v>
       </c>
       <c r="H6" t="str">
-        <v>Approved checkout fixture</v>
+        <v>Start app without payment gateway; use any valid card</v>
       </c>
       <c r="I6" t="str">
-        <v>Implemented</v>
+        <v>To Do</v>
       </c>
       <c r="J6" t="str">
         <v/>
       </c>
       <c r="K6" t="str">
-        <v/>
+        <v>Simulate gateway down by stopping port 4174 before checkout</v>
       </c>
       <c r="L6" t="str">
-        <v/>
+        <v>AI-generated</v>
       </c>
       <c r="M6" t="str">
-        <v>Fallback unless FOODHUB_AI_LIVE=true</v>
+        <v>DeepSeek</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>AI-MISS-001</v>
+        <v>FH-MISS-002</v>
       </c>
       <c r="B7" t="str">
         <v>Missing Scenario</v>
       </c>
       <c r="C7" t="str">
-        <v>Order</v>
+        <v>Observability</v>
       </c>
       <c r="D7" t="str">
-        <v>Duplicate items are submitted as separate order lines</v>
+        <v>Verify request logger writes structured log entry for POST /order</v>
       </c>
       <c r="E7" t="str">
-        <v>Duplicate lines can expose total-calculation mistakes</v>
+        <v>Missing observability data for order creation events, hampering debugging</v>
       </c>
       <c r="F7" t="str">
         <v>Integration</v>
       </c>
       <c r="G7" t="str">
-        <v>Submit the same menu item twice and verify totals remain correct</v>
+        <v>Log file contains entry with method POST, path /order, statusCode 201/400/402, durationMs, requestId</v>
       </c>
       <c r="H7" t="str">
-        <v>Duplicate item order builder</v>
+        <v>Send valid order; check qa-artifacts/observability/raw/request-logs.jsonl</v>
       </c>
       <c r="I7" t="str">
-        <v>Implemented</v>
+        <v>To Do</v>
       </c>
       <c r="J7" t="str">
         <v/>
       </c>
       <c r="K7" t="str">
-        <v/>
+        <v>Run test with NODE_ENV not 'test' to enable logger</v>
       </c>
       <c r="L7" t="str">
-        <v/>
+        <v>AI-generated</v>
       </c>
       <c r="M7" t="str">
-        <v>Fallback unless FOODHUB_AI_LIVE=true</v>
+        <v>DeepSeek</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>AI-MISS-002</v>
+        <v>FH-MISS-003</v>
       </c>
       <c r="B8" t="str">
         <v>Missing Scenario</v>
       </c>
       <c r="C8" t="str">
-        <v>Order</v>
+        <v>Payment</v>
       </c>
       <c r="D8" t="str">
-        <v>Large order at maximum accepted quantity</v>
+        <v>POST /order with invalid payment token format (e.g., 'invalid')</v>
       </c>
       <c r="E8" t="str">
-        <v>Boundary quantities can break validation or totals</v>
+        <v>Payment service may throw unexpected error or not return 402</v>
       </c>
       <c r="F8" t="str">
         <v>Integration</v>
       </c>
       <c r="G8" t="str">
-        <v>Submit quantity 20 and verify the order is accepted with correct total</v>
+        <v>Response status 402 with error 'Payment failed' and details message</v>
       </c>
       <c r="H8" t="str">
-        <v>Boundary quantity order builder</v>
+        <v>Payload with paymentToken: 'invalid'</v>
       </c>
       <c r="I8" t="str">
-        <v>Implemented</v>
+        <v>To Do</v>
       </c>
       <c r="J8" t="str">
         <v/>
       </c>
       <c r="K8" t="str">
-        <v/>
+        <v>FakePaymentGateway returns failed if token does not start with 'gateway_paid_' or 'tok_success'</v>
       </c>
       <c r="L8" t="str">
-        <v/>
+        <v>AI-generated</v>
       </c>
       <c r="M8" t="str">
-        <v>Fallback unless FOODHUB_AI_LIVE=true</v>
+        <v>DeepSeek</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>AI-MISS-003</v>
+        <v>FH-MISS-004</v>
       </c>
       <c r="B9" t="str">
         <v>Missing Scenario</v>
       </c>
       <c r="C9" t="str">
-        <v>Order</v>
+        <v>Persistence</v>
       </c>
       <c r="D9" t="str">
-        <v>Invalid payload shapes are rejected predictably</v>
+        <v>Verify paid order is persisted and retrievable from PostgreSQL via Testcontainers</v>
       </c>
       <c r="E9" t="str">
-        <v>Malformed clients should receive predictable errors</v>
+        <v>Order data may not be saved, leading to loss of transaction records</v>
       </c>
       <c r="F9" t="str">
-        <v>Integration</v>
+        <v>Integration (Testcontainers)</v>
       </c>
       <c r="G9" t="str">
-        <v>Submit items as an object instead of an array and verify 400 response</v>
+        <v>After successful POST /order, query database returns saved receipt with same orderId</v>
       </c>
       <c r="H9" t="str">
-        <v>Malformed payload fixture</v>
+        <v>Real PostgreSQL container; insert order, then read back</v>
       </c>
       <c r="I9" t="str">
-        <v>Implemented</v>
+        <v>To Do</v>
       </c>
       <c r="J9" t="str">
         <v/>
       </c>
       <c r="K9" t="str">
-        <v/>
+        <v>Requires OrderRepository with save method; must be implemented and tested</v>
       </c>
       <c r="L9" t="str">
-        <v/>
+        <v>AI-generated</v>
       </c>
       <c r="M9" t="str">
-        <v>Fallback unless FOODHUB_AI_LIVE=true</v>
+        <v>DeepSeek</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>AI-COV-001</v>
+        <v>FH-EXPN-001</v>
       </c>
       <c r="B10" t="str">
         <v>Coverage Expansion</v>
       </c>
       <c r="C10" t="str">
-        <v>Payment</v>
+        <v>API</v>
       </c>
       <c r="D10" t="str">
-        <v>Gateway cancellation should not create paid orders</v>
+        <v>POST /order with all available menu items in a single order</v>
       </c>
       <c r="E10" t="str">
-        <v>Cancelled payments must not create orders</v>
+        <v>Total calculation may overflow or misbehave with many line items</v>
       </c>
       <c r="F10" t="str">
-        <v>E2E</v>
+        <v>Integration</v>
       </c>
       <c r="G10" t="str">
-        <v>Cancel gateway flow and verify no order is created</v>
+        <v>Status 201 with correct total sum of all items prices times quantities (each quantity 1)</v>
       </c>
       <c r="H10" t="str">
-        <v>Cancelled checkout fixture</v>
+        <v>Payload with items array containing every menu item id with quantity 1</v>
       </c>
       <c r="I10" t="str">
-        <v>Candidate</v>
+        <v>To Do</v>
       </c>
       <c r="J10" t="str">
         <v/>
       </c>
       <c r="K10" t="str">
-        <v/>
+        <v>Ensures pricing logic handles full menu</v>
       </c>
       <c r="L10" t="str">
-        <v/>
+        <v>AI-generated</v>
       </c>
       <c r="M10" t="str">
-        <v>Fallback unless FOODHUB_AI_LIVE=true</v>
+        <v>DeepSeek</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>AI-COV-002</v>
+        <v>FH-EXPN-002</v>
       </c>
       <c r="B11" t="str">
         <v>Coverage Expansion</v>
       </c>
       <c r="C11" t="str">
-        <v>Observability</v>
+        <v>Visual</v>
       </c>
       <c r="D11" t="str">
-        <v>Dashboard refresh and truncate controls have script-level verification</v>
+        <v>Visual regression test on mobile viewport (iPhone 12)</v>
       </c>
       <c r="E11" t="str">
-        <v>Observability drift</v>
+        <v>UI may break on smaller screens, text overflow, layout shift</v>
       </c>
       <c r="F11" t="str">
-        <v>Report</v>
+        <v>E2E (Playwright)</v>
       </c>
       <c r="G11" t="str">
-        <v>Refresh Firebase-backed dashboard and verify generated workbook sheets</v>
+        <v>Screenshots match baseline for menu, cart, and gateway states on mobile</v>
       </c>
       <c r="H11" t="str">
-        <v>Observability metrics fixture</v>
+        <v>Use Playwright device emulation for iPhone 12</v>
       </c>
       <c r="I11" t="str">
-        <v>Implemented</v>
+        <v>To Do</v>
       </c>
       <c r="J11" t="str">
         <v/>
       </c>
       <c r="K11" t="str">
-        <v/>
+        <v>Add new snapshot files for mobile</v>
       </c>
       <c r="L11" t="str">
-        <v/>
+        <v>AI-generated</v>
       </c>
       <c r="M11" t="str">
-        <v>Fallback unless FOODHUB_AI_LIVE=true</v>
+        <v>DeepSeek</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>AI-COV-003</v>
+        <v>FH-EXPN-003</v>
       </c>
       <c r="B12" t="str">
         <v>Coverage Expansion</v>
@@ -1030,59 +1067,210 @@
         <v>Load</v>
       </c>
       <c r="D12" t="str">
-        <v>API handles repeated browse-and-order traffic</v>
+        <v>Load test with 50 concurrent virtual users creating orders</v>
       </c>
       <c r="E12" t="str">
-        <v>Performance regression</v>
+        <v>System may exceed p95 latency or failure thresholds under high concurrency</v>
       </c>
       <c r="F12" t="str">
-        <v>Load</v>
+        <v>Load (k6)</v>
       </c>
       <c r="G12" t="str">
-        <v>k6 thresholds pass for p95 latency, HTTP failures, and paid-order failures</v>
+        <v>http_req_failed rate &lt; 0.05, p95 latency &lt; 500ms, foodhub_order_failures rate &lt; 0.02</v>
       </c>
       <c r="H12" t="str">
-        <v>k6 seeded load data</v>
+        <v>Set VUS=50, ramp-up 30s, steady 60s; use random order templates</v>
       </c>
       <c r="I12" t="str">
-        <v>Implemented</v>
+        <v>To Do</v>
       </c>
       <c r="J12" t="str">
         <v/>
       </c>
       <c r="K12" t="str">
-        <v/>
+        <v>Run after ensuring API and gateway are on HOST=0.0.0.0</v>
       </c>
       <c r="L12" t="str">
-        <v/>
+        <v>AI-generated</v>
       </c>
       <c r="M12" t="str">
-        <v>Fallback unless FOODHUB_AI_LIVE=true</v>
+        <v>DeepSeek</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>FH-EXPN-004</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Coverage Expansion</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Contract</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Pact contract test verifying consumer (Web UI) can consume provider (API) endpoints correctly</v>
+      </c>
+      <c r="E13" t="str">
+        <v>API contract regressions not detected during CI if only integration tests run</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Contract (Pact)</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Pact verification passes for all interactions defined in consumer tests</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Define Pact interactions for menu and order endpoints; provider state setup</v>
+      </c>
+      <c r="I13" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v>Implementation detail: use @pact-foundation/pact</v>
+      </c>
+      <c r="L13" t="str">
+        <v>AI-generated</v>
+      </c>
+      <c r="M13" t="str">
+        <v>DeepSeek</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>FH-EXPN-005</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Coverage Expansion</v>
+      </c>
+      <c r="C14" t="str">
+        <v>AI Recommendation</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Verify aiSuggestion is empty or defaults when cart is empty or consists only of drinks</v>
+      </c>
+      <c r="E14" t="str">
+        <v>AI suggestion logic may generate weird recommendations for edge cases</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Unit/Integration</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Recommended string is sensible and not empty for standard orders; for empty cart or drinks-only, suggestion may be absent or generic</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Order with only drink items (e.g., cola-zero, lemonade)</v>
+      </c>
+      <c r="I14" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v>Check recommendationService logic in src/services/recommendationService.ts</v>
+      </c>
+      <c r="L14" t="str">
+        <v>AI-generated</v>
+      </c>
+      <c r="M14" t="str">
+        <v>DeepSeek</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>FH-EXPN-006</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Coverage Expansion</v>
+      </c>
+      <c r="C15" t="str">
+        <v>UI</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Checkout button disabled state when cart is empty</v>
+      </c>
+      <c r="E15" t="str">
+        <v>User may be able to click checkout with empty cart if button enabled incorrectly</v>
+      </c>
+      <c r="F15" t="str">
+        <v>E2E</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Checkout button should be disabled and have aria-disabled attribute</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Navigate to page with empty cart</v>
+      </c>
+      <c r="I15" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v>Use expect(page.locator('#checkout-button')).toBeDisabled()</v>
+      </c>
+      <c r="L15" t="str">
+        <v>AI-generated</v>
+      </c>
+      <c r="M15" t="str">
+        <v>DeepSeek</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>FH-MISS-005</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Missing Scenario</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Invoice</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Invoice link not available after page refresh mid-session</v>
+      </c>
+      <c r="E16" t="str">
+        <v>User loses ability to view invoice after browser refresh since state is stored in memory only</v>
+      </c>
+      <c r="F16" t="str">
+        <v>E2E</v>
+      </c>
+      <c r="G16" t="str">
+        <v>After refresh, invoice link panel should be hidden (no invoice state persisted); user may need to re-order to see invoice</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Complete an order, then refresh the page; verify invoice link not present</v>
+      </c>
+      <c r="I16" t="str">
+        <v>To Do</v>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v>Not a bug but a UX gap; consider persisting last invoice in localStorage</v>
+      </c>
+      <c r="L16" t="str">
+        <v>AI-generated</v>
+      </c>
+      <c r="M16" t="str">
+        <v>DeepSeek</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M16"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K7"/>
-  <cols>
-    <col min="1" max="1" width="13.83203125" customWidth="1"/>
-    <col min="2" max="2" width="13.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="39.83203125" customWidth="1"/>
-    <col min="6" max="6" width="43.83203125" customWidth="1"/>
-    <col min="7" max="7" width="56.83203125" customWidth="1"/>
-    <col min="8" max="8" width="34.83203125" customWidth="1"/>
-    <col min="9" max="9" width="13.83203125" customWidth="1"/>
-    <col min="10" max="10" width="15.83203125" customWidth="1"/>
-    <col min="11" max="11" width="38.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:K12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1121,217 +1309,392 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>AI-DATA-001</v>
+        <v>TD-001</v>
       </c>
       <c r="B2" t="str">
-        <v>AI-EDGE-004</v>
+        <v>EDGE-001</v>
       </c>
       <c r="C2" t="str">
         <v>Edge Case</v>
       </c>
       <c r="D2" t="str">
-        <v>Randomized mixed order</v>
+        <v>Order payload</v>
       </c>
       <c r="E2" t="str">
-        <v>createRandomOrder(seed)</v>
+        <v>createOrder with quantity 1</v>
       </c>
       <c r="F2" t="str">
-        <v>Seeded deterministic mixed menu items</v>
+        <v>{"items":[{"menuItemId":"burger-classic","quantity":1}],"paymentToken":"gateway_paid_test123","customerName":"Test"}</v>
       </c>
       <c r="G2" t="str">
-        <v>Broaden order combinations without shared mutable data</v>
+        <v>Verify that the minimum valid quantity (1) is accepted and correctly priced</v>
       </c>
       <c r="H2" t="str">
-        <v>Mixed-quantity total validation</v>
+        <v>Integration test</v>
       </c>
       <c r="I2" t="str">
-        <v>Implemented</v>
+        <v>suggested</v>
       </c>
       <c r="J2" t="str">
-        <v/>
+        <v>Manual analysis</v>
       </c>
       <c r="K2" t="str">
-        <v>Fallback unless FOODHUB_AI_LIVE=true</v>
+        <v>N/A</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>AI-DATA-002</v>
+        <v>TD-002</v>
       </c>
       <c r="B3" t="str">
-        <v>AI-MISS-002</v>
+        <v>EDGE-002</v>
       </c>
       <c r="C3" t="str">
-        <v>Missing Scenario</v>
+        <v>Edge Case</v>
       </c>
       <c r="D3" t="str">
-        <v>Boundary quantity</v>
+        <v>Order payload</v>
       </c>
       <c r="E3" t="str">
-        <v>createBoundaryQuantityOrder(20)</v>
+        <v>createBoundaryQuantityOrder(20) (already exists)</v>
       </c>
       <c r="F3" t="str">
-        <v>burger-classic x 20</v>
+        <v>{"items":[{"menuItemId":"burger-classic","quantity":20}],"paymentToken":"gateway_paid_test456","customerName":"Boundary"}</v>
       </c>
       <c r="G3" t="str">
-        <v>Validate upper accepted quantity</v>
+        <v>Confirm boundary quantity 20 is accepted and total is correct (already covered by existing test, listed for completeness)</v>
       </c>
       <c r="H3" t="str">
-        <v>Large order missing scenario</v>
+        <v>Integration test</v>
       </c>
       <c r="I3" t="str">
-        <v>Implemented</v>
+        <v>covered</v>
       </c>
       <c r="J3" t="str">
-        <v/>
+        <v>Existing test</v>
       </c>
       <c r="K3" t="str">
-        <v>Fallback unless FOODHUB_AI_LIVE=true</v>
+        <v>N/A</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>AI-DATA-003</v>
+        <v>TD-003</v>
       </c>
       <c r="B4" t="str">
-        <v>AI-MISS-001</v>
+        <v>MISS-001</v>
       </c>
       <c r="C4" t="str">
         <v>Missing Scenario</v>
       </c>
       <c r="D4" t="str">
-        <v>Duplicate item lines</v>
+        <v>Payment token</v>
       </c>
       <c r="E4" t="str">
-        <v>createDuplicateItemOrder()</v>
+        <v>createOrder with paymentToken "tok_success"</v>
       </c>
       <c r="F4" t="str">
-        <v>burger-classic x 1 and burger-classic x 2</v>
+        <v>{"items":[{"menuItemId":"lemonade","quantity":2}],"paymentToken":"tok_success","customerName":"TokenSuccess"}</v>
       </c>
       <c r="G4" t="str">
-        <v>Validate totals across repeated menu item ids</v>
+        <v>Test that the legacy success token 'tok_success' is handled correctly and returns a paid receipt</v>
       </c>
       <c r="H4" t="str">
-        <v>Duplicate items missing scenario</v>
+        <v>Integration test</v>
       </c>
       <c r="I4" t="str">
-        <v>Implemented</v>
+        <v>suggested</v>
       </c>
       <c r="J4" t="str">
-        <v/>
+        <v>Code review – paymentService accepts 'tok_success' but no integration test uses it</v>
       </c>
       <c r="K4" t="str">
-        <v>Fallback unless FOODHUB_AI_LIVE=true</v>
+        <v>N/A</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>AI-DATA-004</v>
+        <v>TD-004</v>
       </c>
       <c r="B5" t="str">
-        <v>AI-EDGE-005</v>
+        <v>MISS-002</v>
       </c>
       <c r="C5" t="str">
-        <v>Edge Case</v>
+        <v>Missing Scenario</v>
       </c>
       <c r="D5" t="str">
-        <v>Invoice customer</v>
+        <v>Order payload</v>
       </c>
       <c r="E5" t="str">
-        <v>createApprovedCheckout().customerName</v>
+        <v>createOrder with customerName set to whitespace-only string</v>
       </c>
       <c r="F5" t="str">
-        <v>FoodHub Demo User</v>
+        <v>{"items":[{"menuItemId":"wrap-veggie","quantity":1}],"paymentToken":"gateway_paid_test789","customerName":"   "}</v>
       </c>
       <c r="G5" t="str">
-        <v>Verify invoice customer-name publishing</v>
+        <v>Ensure that a customerName consisting only of whitespace is rejected (Zod .trim().min(1))</v>
       </c>
       <c r="H5" t="str">
-        <v>Invoice receipt validation</v>
+        <v>Integration test</v>
       </c>
       <c r="I5" t="str">
-        <v>Implemented</v>
+        <v>suggested</v>
       </c>
       <c r="J5" t="str">
-        <v/>
+        <v>Code analysis – schema uses .trim().min(1) but not tested</v>
       </c>
       <c r="K5" t="str">
-        <v>Fallback unless FOODHUB_AI_LIVE=true</v>
+        <v>N/A</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>AI-DATA-005</v>
+        <v>TD-005</v>
       </c>
       <c r="B6" t="str">
-        <v>AI-COV-003</v>
+        <v>EDGE-003</v>
       </c>
       <c r="C6" t="str">
-        <v>Coverage Expansion</v>
+        <v>Edge Case</v>
       </c>
       <c r="D6" t="str">
-        <v>Load traffic</v>
+        <v>Order payload</v>
       </c>
       <c r="E6" t="str">
-        <v>k6 __VU/__ITER payment token</v>
+        <v>createOrder with quantity 0</v>
       </c>
       <c r="F6" t="str">
-        <v>gateway_paid_load_1_1</v>
+        <v>{"items":[{"menuItemId":"burger-classic","quantity":0}],"paymentToken":"gateway_paid_test000","customerName":"ZeroQty"}</v>
       </c>
       <c r="G6" t="str">
-        <v>Avoid payment-token collisions during load execution</v>
+        <v>Verify that quantity 0 is rejected (z.number().int().positive())</v>
       </c>
       <c r="H6" t="str">
-        <v>Load coverage expansion</v>
+        <v>Integration test</v>
       </c>
       <c r="I6" t="str">
-        <v>Implemented</v>
+        <v>suggested</v>
       </c>
       <c r="J6" t="str">
-        <v/>
+        <v>Manual analysis – positive constraint not covered</v>
       </c>
       <c r="K6" t="str">
-        <v>Fallback unless FOODHUB_AI_LIVE=true</v>
+        <v>N/A</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>AI-DATA-006</v>
+        <v>TD-006</v>
       </c>
       <c r="B7" t="str">
-        <v>AI-COV-002</v>
+        <v>EDGE-004</v>
       </c>
       <c r="C7" t="str">
+        <v>Edge Case</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Order payload</v>
+      </c>
+      <c r="E7" t="str">
+        <v>createOrder with negative quantity</v>
+      </c>
+      <c r="F7" t="str">
+        <v>{"items":[{"menuItemId":"cola-zero","quantity":-3}],"paymentToken":"gateway_paid_test111","customerName":"NegativeQty"}</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Ensure negative quantity is rejected by Zod or validation logic</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Integration test</v>
+      </c>
+      <c r="I7" t="str">
+        <v>suggested</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Manual analysis – negative integer not tested</v>
+      </c>
+      <c r="K7" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TD-007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>MISS-003</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Missing Scenario</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Order payload</v>
+      </c>
+      <c r="E8" t="str">
+        <v>createOrder with null items element</v>
+      </c>
+      <c r="F8" t="str">
+        <v>{"items":[null],"paymentToken":"gateway_paid_test222","customerName":"NullItem"}</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Check that an array containing null is rejected with 400 error</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Integration test</v>
+      </c>
+      <c r="I8" t="str">
+        <v>suggested</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Code review – Zod array of objects, null element not tested</v>
+      </c>
+      <c r="K8" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TD-008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>COV-001</v>
+      </c>
+      <c r="C9" t="str">
         <v>Coverage Expansion</v>
       </c>
-      <c r="D7" t="str">
-        <v>Observability metrics</v>
-      </c>
-      <c r="E7" t="str">
-        <v>latest-observability-metrics.json</v>
-      </c>
-      <c r="F7" t="str">
-        <v>requestCount, errorCount, p95DurationMs</v>
-      </c>
-      <c r="G7" t="str">
-        <v>Feed Firebase and charted dashboard</v>
-      </c>
-      <c r="H7" t="str">
-        <v>Observability coverage expansion</v>
-      </c>
-      <c r="I7" t="str">
-        <v>Implemented</v>
-      </c>
-      <c r="J7" t="str">
-        <v/>
-      </c>
-      <c r="K7" t="str">
-        <v>Fallback unless FOODHUB_AI_LIVE=true</v>
+      <c r="D9" t="str">
+        <v>Order payload</v>
+      </c>
+      <c r="E9" t="str">
+        <v>createRandomOrder(10) or a new builder createLargeDistinctOrder</v>
+      </c>
+      <c r="F9" t="str">
+        <v>{"items":[{"menuItemId":"burger-classic","quantity":1},{"menuItemId":"wrap-veggie","quantity":2},{"menuItemId":"lemonade","quantity":1},{"menuItemId":"cola-zero","quantity":1},{"menuItemId":"fries-large","quantity":1}],"paymentToken":"gateway_paid_test333","customerName":"LargeOrder"}</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Verify that an order with many unique items (e.g., 5+ distinct menu items) processes correctly and total is accurate</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Integration test / Load test</v>
+      </c>
+      <c r="I9" t="str">
+        <v>suggested</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Coverage analysis – only small orders tested</v>
+      </c>
+      <c r="K9" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TD-009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>COV-002</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Coverage Expansion</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Order payload</v>
+      </c>
+      <c r="E10" t="str">
+        <v>createOrder with a price that causes floating point rounding</v>
+      </c>
+      <c r="F10" t="str">
+        <v>{"items":[{"menuItemId":"items with price 0.10","quantity":3}],"paymentToken":"gateway_paid_test444","customerName":"RoundingTest"}</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Ensure roundMoney correctly handles floating point arithmetic (e.g., 0.10 * 3 = 0.30, not 0.30000000000000004)</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Integration test</v>
+      </c>
+      <c r="I10" t="str">
+        <v>suggested</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Code analysis – roundMoney uses Number.EPSILON, no explicit test</v>
+      </c>
+      <c r="K10" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>TD-010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>MISS-004</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Missing Scenario</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Payment token</v>
+      </c>
+      <c r="E11" t="str">
+        <v>createOrder with paymentToken missing from request</v>
+      </c>
+      <c r="F11" t="str">
+        <v>{"items":[{"menuItemId":"fries-large","quantity":1}],"customerName":"NoToken"}</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Validate that a missing paymentToken field is caught by Zod (z.string().min(1)) and returns 400</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Integration test</v>
+      </c>
+      <c r="I11" t="str">
+        <v>suggested</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Manual analysis – required field not tested for absence</v>
+      </c>
+      <c r="K11" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>TD-011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>EDGE-005</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Edge Case</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Order payload</v>
+      </c>
+      <c r="E12" t="str">
+        <v>createOrder with customerName of length 255</v>
+      </c>
+      <c r="F12" t="str">
+        <v>{"items":[{"menuItemId":"burger-classic","quantity":1}],"paymentToken":"gateway_paid_test555","customerName":"a... (255 characters)"}</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Test that a very long customerName (255 chars) is accepted or rejected appropriately (no length constraint in schema, but may cause DB issues)</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Integration test</v>
+      </c>
+      <c r="I12" t="str">
+        <v>suggested</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Edge case analysis – no length validation on customerName</v>
+      </c>
+      <c r="K12" t="str">
+        <v>N/A</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1340,9 +1703,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C7"/>
   <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
-    <col min="2" max="2" width="47.83203125" customWidth="1"/>
-    <col min="3" max="3" width="64.83203125" customWidth="1"/>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="90.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1372,7 +1735,7 @@
         <v>DeepSeek API key</v>
       </c>
       <c r="B3" t="str">
-        <v>Not configured</v>
+        <v>Configured</v>
       </c>
       <c r="C3" t="str">
         <v>DeepSeek bearer token loaded from Firestore foodhub-6ba1c/deepSeek/ooz80WHRgmUV3WseQDnF/api-key</v>

</xml_diff>